<commit_message>
Add prices in USD to Regal_URLs.xlsx
</commit_message>
<xml_diff>
--- a/Regal Collection Images/Regal_URLs.xlsx
+++ b/Regal Collection Images/Regal_URLs.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regal Collection URLs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regal Collection" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="5">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+  </numFmts>
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,8 +45,15 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <color rgb="00C00000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +63,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002C3E50"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF99"/>
       </patternFill>
     </fill>
   </fills>
@@ -82,15 +97,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -456,13 +484,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="95" customWidth="1" min="3" max="3"/>
-    <col width="95" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="95" customWidth="1" min="5" max="5"/>
+    <col width="95" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -478,10 +508,20 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Price (USD)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Production Days</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Landscape (full image)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Portrait (main image)</t>
         </is>
@@ -498,12 +538,22 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/REGAL%20COLLECTION.jpg</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -520,12 +570,20 @@
           <t>R1021</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="6" t="n">
+        <v>2580</v>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/REGINA.jpg</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/REGINA.jpg</t>
         </is>
@@ -542,12 +600,20 @@
           <t>R1022</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="6" t="n">
+        <v>2450</v>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/ELARION.jpg</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/ELARION.jpg</t>
         </is>
@@ -564,12 +630,20 @@
           <t>R1023</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/ODETTE.jpg</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/ODETTE.jpg</t>
         </is>
@@ -586,12 +660,20 @@
           <t>R1024</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="6" t="n">
+        <v>1950</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/EVANGELINE.jpg</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/EVANGELINE.jpg</t>
         </is>
@@ -608,12 +690,20 @@
           <t>R1025</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="6" t="n">
+        <v>1950</v>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/ROSALINE.jpg</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/ROSALINE.jpg</t>
         </is>
@@ -630,12 +720,20 @@
           <t>R1026</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="6" t="n">
+        <v>2250</v>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/CORNELIA.jpg</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/CORNELIA.jpg</t>
         </is>
@@ -652,12 +750,20 @@
           <t>R1027</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="6" t="n">
+        <v>2450</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/MIRAVELLE.jpg</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/MIRAVELLE.jpg</t>
         </is>
@@ -674,12 +780,20 @@
           <t>R1028</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="6" t="n">
+        <v>1950</v>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/VALTORIA.jpg</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/VALTORIA.jpg</t>
         </is>
@@ -696,12 +810,20 @@
           <t>R1029</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="6" t="n">
+        <v>2850</v>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/VESPERA.jpg</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/VESPERA.jpg</t>
         </is>
@@ -718,12 +840,20 @@
           <t>R1030</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="6" t="n">
+        <v>2850</v>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/AURETTE.jpg</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/AURETTE.jpg</t>
         </is>
@@ -740,12 +870,20 @@
           <t>R1031</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="6" t="n">
+        <v>1700</v>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/ISALINE.jpg</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/ISALINE.jpg</t>
         </is>
@@ -762,12 +900,20 @@
           <t>R1032</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="6" t="n">
+        <v>1950</v>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/ALOUETTE.jpg</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/ALOUETTE.jpg</t>
         </is>
@@ -784,12 +930,20 @@
           <t>R1033</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="6" t="n">
+        <v>1700</v>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/NORIELLE.jpg</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/NORIELLE.jpg</t>
         </is>
@@ -806,12 +960,20 @@
           <t>R1034</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="6" t="n">
+        <v>2850</v>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/VIVIENNE.jpg</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/VIVIENNE.jpg</t>
         </is>
@@ -828,12 +990,20 @@
           <t>R1035</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="6" t="n">
+        <v>1950</v>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/ALTHEA.jpg</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/ALTHEA.jpg</t>
         </is>
@@ -850,12 +1020,20 @@
           <t>R1036</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" s="6" t="n">
+        <v>2250</v>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/SABINE.jpg</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/SABINE.jpg</t>
         </is>
@@ -872,12 +1050,20 @@
           <t>R1037</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="6" t="n">
+        <v>1700</v>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/CLARISSE.jpg</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/CLARISSE.jpg</t>
         </is>
@@ -894,12 +1080,20 @@
           <t>R1038</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="6" t="n">
+        <v>2600</v>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/MATILDA.jpg</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/MATILDA.jpg</t>
         </is>
@@ -916,12 +1110,20 @@
           <t>R1039</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C21" s="6" t="n">
+        <v>2850</v>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/MARQUISE.jpg</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/MARQUISE.jpg</t>
         </is>
@@ -938,60 +1140,103 @@
           <t>R1040</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C22" s="6" t="n">
+        <v>1950</v>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/LUNARA.jpg</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/LUNARA.jpg</t>
         </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Collection order</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="n">
+        <v>44780</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Discount</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="n">
+        <v>-3582.4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>TOTAL (Mix Collection, 20 dresses)</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="n">
+        <v>41197.6</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId41"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Silhouette column to Regal_URLs.xlsx
</commit_message>
<xml_diff>
--- a/Regal Collection Images/Regal_URLs.xlsx
+++ b/Regal Collection Images/Regal_URLs.xlsx
@@ -53,7 +53,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -63,6 +63,31 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002C3E50"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F4FD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEBEE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3E5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3E0"/>
       </patternFill>
     </fill>
     <fill>
@@ -97,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -108,7 +133,22 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -118,7 +158,7 @@
     </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -484,15 +524,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="95" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="95" customWidth="1" min="6" max="6"/>
+    <col width="95" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -508,20 +549,25 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Silhouette</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Price (USD)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Production Days</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Landscape (full image)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Portrait (main image)</t>
         </is>
@@ -548,12 +594,17 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/REGAL%20COLLECTION.jpg</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -570,20 +621,25 @@
           <t>R1021</t>
         </is>
       </c>
-      <c r="C3" s="6" t="n">
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>A-LINE</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="n">
         <v>2580</v>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>30-120</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/REGINA.jpg</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/REGINA.jpg</t>
         </is>
@@ -600,20 +656,25 @@
           <t>R1022</t>
         </is>
       </c>
-      <c r="C4" s="6" t="n">
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>BALL GOWN</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="n">
         <v>2450</v>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>30-120</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/ELARION.jpg</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/ELARION.jpg</t>
         </is>
@@ -630,20 +691,25 @@
           <t>R1023</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>MINI</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="n">
         <v>2000</v>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>30-120</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/ODETTE.jpg</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/ODETTE.jpg</t>
         </is>
@@ -660,20 +726,25 @@
           <t>R1024</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>A-LINE</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="n">
         <v>1950</v>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>30-120</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/EVANGELINE.jpg</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/EVANGELINE.jpg</t>
         </is>
@@ -690,20 +761,25 @@
           <t>R1025</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>A-LINE</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="n">
         <v>1950</v>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>30-120</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/ROSALINE.jpg</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/ROSALINE.jpg</t>
         </is>
@@ -720,20 +796,25 @@
           <t>R1026</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>A-LINE</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="n">
         <v>2250</v>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>30-120</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/CORNELIA.jpg</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/CORNELIA.jpg</t>
         </is>
@@ -750,20 +831,25 @@
           <t>R1027</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>BALL GOWN</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="n">
         <v>2450</v>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>30-120</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/MIRAVELLE.jpg</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/MIRAVELLE.jpg</t>
         </is>
@@ -780,20 +866,25 @@
           <t>R1028</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>A-LINE</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="n">
         <v>1950</v>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>30-120</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/VALTORIA.jpg</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/VALTORIA.jpg</t>
         </is>
@@ -810,20 +901,25 @@
           <t>R1029</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>BALL GOWN</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="n">
         <v>2850</v>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>30-120</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/VESPERA.jpg</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/VESPERA.jpg</t>
         </is>
@@ -840,20 +936,25 @@
           <t>R1030</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>SHEATH</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="n">
         <v>2850</v>
       </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>30-120</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/AURETTE.jpg</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/AURETTE.jpg</t>
         </is>
@@ -870,20 +971,25 @@
           <t>R1031</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>A-LINE</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="n">
         <v>1700</v>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>30-120</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/ISALINE.jpg</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/ISALINE.jpg</t>
         </is>
@@ -900,20 +1006,25 @@
           <t>R1032</t>
         </is>
       </c>
-      <c r="C14" s="6" t="n">
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>A-LINE</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="n">
         <v>1950</v>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>30-120</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/ALOUETTE.jpg</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/ALOUETTE.jpg</t>
         </is>
@@ -930,20 +1041,25 @@
           <t>R1033</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n">
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>A-LINE</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="n">
         <v>1700</v>
       </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>30-120</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/NORIELLE.jpg</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/NORIELLE.jpg</t>
         </is>
@@ -960,20 +1076,25 @@
           <t>R1034</t>
         </is>
       </c>
-      <c r="C16" s="6" t="n">
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>A-LINE</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="n">
         <v>2850</v>
       </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>30-120</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/VIVIENNE.jpg</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/VIVIENNE.jpg</t>
         </is>
@@ -990,20 +1111,25 @@
           <t>R1035</t>
         </is>
       </c>
-      <c r="C17" s="6" t="n">
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>BALL GOWN</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="n">
         <v>1950</v>
       </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>30-120</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/ALTHEA.jpg</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/ALTHEA.jpg</t>
         </is>
@@ -1020,20 +1146,25 @@
           <t>R1036</t>
         </is>
       </c>
-      <c r="C18" s="6" t="n">
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>MERMAID</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="n">
         <v>2250</v>
       </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>30-120</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/SABINE.jpg</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/SABINE.jpg</t>
         </is>
@@ -1050,20 +1181,25 @@
           <t>R1037</t>
         </is>
       </c>
-      <c r="C19" s="6" t="n">
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>MINI</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="n">
         <v>1700</v>
       </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>30-120</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/CLARISSE.jpg</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/CLARISSE.jpg</t>
         </is>
@@ -1080,20 +1216,25 @@
           <t>R1038</t>
         </is>
       </c>
-      <c r="C20" s="6" t="n">
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>MERMAID</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="n">
         <v>2600</v>
       </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>30-120</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/MATILDA.jpg</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/MATILDA.jpg</t>
         </is>
@@ -1110,20 +1251,25 @@
           <t>R1039</t>
         </is>
       </c>
-      <c r="C21" s="6" t="n">
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>A-LINE</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="n">
         <v>2850</v>
       </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>30-120</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/MARQUISE.jpg</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/MARQUISE.jpg</t>
         </is>
@@ -1140,103 +1286,108 @@
           <t>R1040</t>
         </is>
       </c>
-      <c r="C22" s="6" t="n">
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>SHEATH</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="n">
         <v>1950</v>
       </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>30-120</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>30-120</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/Regal%20Collection%20Images/LUNARA.jpg</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/idogolan4955/avians-media/main/%D7%AA%D7%9E%D7%95%D7%A0%D7%94%20%D7%A8%D7%90%D7%A9%D7%99%D7%AA/LUNARA.jpg</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>Collection order</t>
         </is>
       </c>
-      <c r="C24" s="8" t="n">
+      <c r="D24" s="13" t="n">
         <v>44780</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>Discount</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>8%</t>
         </is>
       </c>
-      <c r="C25" s="10" t="n">
+      <c r="D25" s="15" t="n">
         <v>-3582.4</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="A26" s="16" t="inlineStr">
         <is>
           <t>TOTAL (Mix Collection, 20 dresses)</t>
         </is>
       </c>
-      <c r="C26" s="12" t="n">
+      <c r="D26" s="17" t="n">
         <v>41197.6</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId41"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>